<commit_message>
vault backup: 2026-10-09 13:19:35
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1452,10 +1452,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F21" s="3">
         <f>IF(OR(E21="",G21&lt;&gt;"",H21&lt;&gt;""),"",WORKDAY(E21,5))</f>
         <v/>
@@ -1474,7 +1476,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>PDF fehlt noch (Codex)</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>
@@ -1496,10 +1498,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F22" s="3">
         <f>IF(OR(E22="",G22&lt;&gt;"",H22&lt;&gt;""),"",WORKDAY(E22,5))</f>
         <v/>
@@ -1518,7 +1522,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>PDF fehlt noch (Codex)</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>
@@ -1540,10 +1544,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F23" s="3">
         <f>IF(OR(E23="",G23&lt;&gt;"",H23&lt;&gt;""),"",WORKDAY(E23,5))</f>
         <v/>
@@ -1562,7 +1568,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>PDF fehlt noch (Codex)</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>
@@ -1584,10 +1590,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F24" s="3">
         <f>IF(OR(E24="",G24&lt;&gt;"",H24&lt;&gt;""),"",WORKDAY(E24,5))</f>
         <v/>
@@ -1606,7 +1614,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>PDF fehlt noch (Codex)</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-09 13:39:51
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1619,10 +1619,26 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>RPGA Design Group</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Architektur</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>rickgarza@rpgaarchitects.com</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3">
         <f>IF(OR(E25="",G25&lt;&gt;"",H25&lt;&gt;""),"",WORKDAY(E25,5))</f>
@@ -1635,14 +1651,38 @@
         <f>IF(A25="","",IF(I25&lt;&gt;"","Antwort bearbeiten",IF(G25&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G25,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E25&lt;&gt;"",IF(TODAY()&gt;=F25,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D25="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>CHS Architects</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Architektur</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>info@chsarchitects.com</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3">
         <f>IF(OR(E26="",G26&lt;&gt;"",H26&lt;&gt;""),"",WORKDAY(E26,5))</f>
@@ -1655,14 +1695,38 @@
         <f>IF(A26="","",IF(I26&lt;&gt;"","Antwort bearbeiten",IF(G26&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G26,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E26&lt;&gt;"",IF(TODAY()&gt;=F26,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D26="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>PDMS Design Group</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Architektur</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>design@pdmsdesign.com</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3">
         <f>IF(OR(E27="",G27&lt;&gt;"",H27&lt;&gt;""),"",WORKDAY(E27,5))</f>
@@ -1675,14 +1739,38 @@
         <f>IF(A27="","",IF(I27&lt;&gt;"","Antwort bearbeiten",IF(G27&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G27,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E27&lt;&gt;"",IF(TODAY()&gt;=F27,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D27="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Touch Ya' Soul Food Catering</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>touchyasoulfoodcatering@gmail.com</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3">
         <f>IF(OR(E28="",G28&lt;&gt;"",H28&lt;&gt;""),"",WORKDAY(E28,5))</f>
@@ -1695,14 +1783,38 @@
         <f>IF(A28="","",IF(I28&lt;&gt;"","Antwort bearbeiten",IF(G28&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G28,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E28&lt;&gt;"",IF(TODAY()&gt;=F28,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D28="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>David's Barbecue</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Gastro</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>austin@davidsbarbecuetx.com</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3">
         <f>IF(OR(E29="",G29&lt;&gt;"",H29&lt;&gt;""),"",WORKDAY(E29,5))</f>
@@ -1715,8 +1827,16 @@
         <f>IF(A29="","",IF(I29&lt;&gt;"","Antwort bearbeiten",IF(G29&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G29,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E29&lt;&gt;"",IF(TODAY()&gt;=F29,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D29="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>

</xml_diff>

<commit_message>
vault backup: 2026-10-09 14:40:26
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1658,7 +1658,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mails Gastro/Architektur (5 Firmen), versandfertig, nicht verschickt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1636,7 +1636,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E25" s="3" t="n"/>
@@ -1653,12 +1653,12 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+          <t>11-Versandfertig-Gastro-Architektur</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E26" s="3" t="n"/>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+          <t>11-Versandfertig-Gastro-Architektur</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E27" s="3" t="n"/>
@@ -1741,12 +1741,12 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+          <t>11-Versandfertig-Gastro-Architektur</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E28" s="3" t="n"/>
@@ -1785,12 +1785,12 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+          <t>11-Versandfertig-Gastro-Architektur</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E29" s="3" t="n"/>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Gastro-Architektur-2026-10-09</t>
+          <t>11-Versandfertig-Gastro-Architektur</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10. (leads/…), Mail und PDF offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-09 18:26:03
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1636,10 +1636,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F25" s="3">
         <f>IF(OR(E25="",G25&lt;&gt;"",H25&lt;&gt;""),"",WORKDAY(E25,5))</f>
         <v/>
@@ -1658,7 +1660,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>
@@ -1680,10 +1682,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F26" s="3">
         <f>IF(OR(E26="",G26&lt;&gt;"",H26&lt;&gt;""),"",WORKDAY(E26,5))</f>
         <v/>
@@ -1702,7 +1706,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>
@@ -1724,10 +1728,12 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F27" s="3">
         <f>IF(OR(E27="",G27&lt;&gt;"",H27&lt;&gt;""),"",WORKDAY(E27,5))</f>
         <v/>
@@ -1746,7 +1752,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>
@@ -1768,10 +1774,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F28" s="3">
         <f>IF(OR(E28="",G28&lt;&gt;"",H28&lt;&gt;""),"",WORKDAY(E28,5))</f>
         <v/>
@@ -1790,7 +1798,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>
@@ -1812,10 +1820,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F29" s="3">
         <f>IF(OR(E29="",G29&lt;&gt;"",H29&lt;&gt;""),"",WORKDAY(E29,5))</f>
         <v/>
@@ -1834,7 +1844,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10.; frühestens 12.10. senden</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Akquise: 5 Gastro/Architektur-Mails als verschickt markiert, neue Service-Leads (Schädlingsbekämpfung, Autowerkstatt, Zahnarzt)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1849,10 +1849,26 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Fort Worth Pest &amp; Termite</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Schädlingsbekämpfung</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>sales@fortworthpest.com</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="n"/>
       <c r="F30" s="3">
         <f>IF(OR(E30="",G30&lt;&gt;"",H30&lt;&gt;""),"",WORKDAY(E30,5))</f>
@@ -1865,14 +1881,38 @@
         <f>IF(A30="","",IF(I30&lt;&gt;"","Antwort bearbeiten",IF(G30&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G30,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E30&lt;&gt;"",IF(TODAY()&gt;=F30,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D30="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="n"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Service-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Mike's Brake &amp; Alignment</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Autowerkstatt</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>mikesbrakeandalignment@gmail.com</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3">
         <f>IF(OR(E31="",G31&lt;&gt;"",H31&lt;&gt;""),"",WORKDAY(E31,5))</f>
@@ -1885,14 +1925,38 @@
         <f>IF(A31="","",IF(I31&lt;&gt;"","Antwort bearbeiten",IF(G31&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G31,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E31&lt;&gt;"",IF(TODAY()&gt;=F31,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D31="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Service-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>BBN Pest Control</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Schädlingsbekämpfung</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>bbnpestcontrol@aol.com</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3">
         <f>IF(OR(E32="",G32&lt;&gt;"",H32&lt;&gt;""),"",WORKDAY(E32,5))</f>
@@ -1905,14 +1969,38 @@
         <f>IF(A32="","",IF(I32&lt;&gt;"","Antwort bearbeiten",IF(G32&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G32,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E32&lt;&gt;"",IF(TODAY()&gt;=F32,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D32="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Service-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Burleson Dental Care</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Zahnarzt</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>info@burlesondentalcare.com</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E33" s="3" t="n"/>
       <c r="F33" s="3">
         <f>IF(OR(E33="",G33&lt;&gt;"",H33&lt;&gt;""),"",WORKDAY(E33,5))</f>
@@ -1925,14 +2013,38 @@
         <f>IF(A33="","",IF(I33&lt;&gt;"","Antwort bearbeiten",IF(G33&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G33,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E33&lt;&gt;"",IF(TODAY()&gt;=F33,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D33="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K33" s="2" t="n"/>
-      <c r="L33" s="2" t="n"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Service-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Chief Pest Control</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Schädlingsbekämpfung</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>chiefpestmail@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3">
         <f>IF(OR(E34="",G34&lt;&gt;"",H34&lt;&gt;""),"",WORKDAY(E34,5))</f>
@@ -1945,8 +2057,16 @@
         <f>IF(A34="","",IF(I34&lt;&gt;"","Antwort bearbeiten",IF(G34&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G34,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E34&lt;&gt;"",IF(TODAY()&gt;=F34,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D34="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Neue-Leads-Service-2026-10-09</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 09.10., Konzept offen</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>

</xml_diff>

<commit_message>
Konzepte Service-Nischen: 4 Konzeptseiten (Mike's, BBN, Fort Worth Pest & Termite, Burleson Dental)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1888,7 +1888,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 09.10., Konzept offen</t>
+          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mails Service-Nischen (4 Firmen) vorbereitet, nicht verschickt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1883,12 +1883,12 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Service-2026-10-09</t>
+          <t>12-Versandfertig-Service</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
+          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
         </is>
       </c>
     </row>
@@ -1927,12 +1927,12 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Service-2026-10-09</t>
+          <t>12-Versandfertig-Service</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
+          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Service-2026-10-09</t>
+          <t>12-Versandfertig-Service</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
+          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
         </is>
       </c>
     </row>
@@ -2015,12 +2015,12 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Neue-Leads-Service-2026-10-09</t>
+          <t>12-Versandfertig-Service</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 09.10., Mail/PDF/Video offen</t>
+          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Service-Leads: PDFs, Scroll-Videos und Ganzseiten-Bilder für Fort Worth Pest & Termite, Mike's, BBN und Burleson Dental; Mails versandbereit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1866,7 +1866,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E30" s="3" t="n"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E31" s="3" t="n"/>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E32" s="3" t="n"/>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E33" s="3" t="n"/>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite und Mail fertig 09.10., PDF/Video offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-10 07:16:57
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1866,10 +1866,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F30" s="3">
         <f>IF(OR(E30="",G30&lt;&gt;"",H30&lt;&gt;""),"",WORKDAY(E30,5))</f>
         <v/>
@@ -1888,7 +1890,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
+          <t>Erstmail 09.10. mit PDF verschickt</t>
         </is>
       </c>
     </row>
@@ -1910,10 +1912,12 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F31" s="3">
         <f>IF(OR(E31="",G31&lt;&gt;"",H31&lt;&gt;""),"",WORKDAY(E31,5))</f>
         <v/>
@@ -1932,7 +1936,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
+          <t>Erstmail 09.10. mit PDF verschickt</t>
         </is>
       </c>
     </row>
@@ -1954,10 +1958,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F32" s="3">
         <f>IF(OR(E32="",G32&lt;&gt;"",H32&lt;&gt;""),"",WORKDAY(E32,5))</f>
         <v/>
@@ -1976,7 +1982,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
+          <t>Erstmail 09.10. mit PDF verschickt</t>
         </is>
       </c>
     </row>
@@ -1998,10 +2004,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>46304</v>
+      </c>
       <c r="F33" s="3">
         <f>IF(OR(E33="",G33&lt;&gt;"",H33&lt;&gt;""),"",WORKDAY(E33,5))</f>
         <v/>
@@ -2020,7 +2028,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 09.10., versandbereit</t>
+          <t>Erstmail 09.10. mit PDF verschickt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Akquise: Service-Mails als verschickt (09.10.) eingetragen, 5 neue Leads in Mix-Nischen (Motorrad, Karosserie, Reinigung, Tanz, Chiropraktik)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2077,10 +2077,26 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Monkey Wrench Cycles</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Motorradwerkstatt</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>FrankV@MonkeyWrenchMotorcycles.com</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3">
         <f>IF(OR(E35="",G35&lt;&gt;"",H35&lt;&gt;""),"",WORKDAY(E35,5))</f>
@@ -2094,13 +2110,33 @@
         <v/>
       </c>
       <c r="K35" s="2" t="n"/>
-      <c r="L35" s="2" t="n"/>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Factory Finish Auto Collision Center</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Karosseriewerkstatt</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>factoryfinishpb@sbcglobal.net</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E36" s="3" t="n"/>
       <c r="F36" s="3">
         <f>IF(OR(E36="",G36&lt;&gt;"",H36&lt;&gt;""),"",WORKDAY(E36,5))</f>
@@ -2114,13 +2150,33 @@
         <v/>
       </c>
       <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Kite's Custom Cleaners</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Reinigung</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>info@kitescleaners.com</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3">
         <f>IF(OR(E37="",G37&lt;&gt;"",H37&lt;&gt;""),"",WORKDAY(E37,5))</f>
@@ -2134,13 +2190,33 @@
         <v/>
       </c>
       <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Studio of MoveMINT</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Tanzschule</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>info@studioofmovemint.com</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3">
         <f>IF(OR(E38="",G38&lt;&gt;"",H38&lt;&gt;""),"",WORKDAY(E38,5))</f>
@@ -2154,13 +2230,33 @@
         <v/>
       </c>
       <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Arlington Natural Wellness Center</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Chiropraktik</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>arlingtonnwc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3">
         <f>IF(OR(E39="",G39&lt;&gt;"",H39&lt;&gt;""),"",WORKDAY(E39,5))</f>
@@ -2174,7 +2270,11 @@
         <v/>
       </c>
       <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="n"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>

</xml_diff>

<commit_message>
vault backup: 2026-10-10 08:37:18
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2112,7 +2112,7 @@
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mix-Leads: Projektnotizen, PDFs, Scroll-Videos und Ganzseiten-Bilder für Monkey Wrench Cycles, Factory Finish, Kite's, Studio of MoveMINT, Arlington Natural Wellness
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2112,7 +2112,7 @@
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mix-Leads: fünf Akquise-Mails vorbereitet (13-Versandfertig-Mix), in den Projektnotizen, Tracker auf Versandbereit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2094,7 +2094,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E35" s="3" t="n"/>
@@ -2109,10 +2109,14 @@
         <f>IF(A35="","",IF(I35&lt;&gt;"","Antwort bearbeiten",IF(G35&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G35,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E35&lt;&gt;"",IF(TODAY()&gt;=F35,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D35="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K35" s="2" t="n"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>13-Versandfertig-Mix</t>
+        </is>
+      </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2138,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E36" s="3" t="n"/>
@@ -2149,10 +2153,14 @@
         <f>IF(A36="","",IF(I36&lt;&gt;"","Antwort bearbeiten",IF(G36&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G36,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E36&lt;&gt;"",IF(TODAY()&gt;=F36,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D36="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K36" s="2" t="n"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>13-Versandfertig-Mix</t>
+        </is>
+      </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2182,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E37" s="3" t="n"/>
@@ -2189,10 +2197,14 @@
         <f>IF(A37="","",IF(I37&lt;&gt;"","Antwort bearbeiten",IF(G37&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G37,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E37&lt;&gt;"",IF(TODAY()&gt;=F37,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D37="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K37" s="2" t="n"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>13-Versandfertig-Mix</t>
+        </is>
+      </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2226,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E38" s="3" t="n"/>
@@ -2229,10 +2241,14 @@
         <f>IF(A38="","",IF(I38&lt;&gt;"","Antwort bearbeiten",IF(G38&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G38,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E38&lt;&gt;"",IF(TODAY()&gt;=F38,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D38="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K38" s="2" t="n"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>13-Versandfertig-Mix</t>
+        </is>
+      </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2270,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E39" s="3" t="n"/>
@@ -2269,10 +2285,14 @@
         <f>IF(A39="","",IF(I39&lt;&gt;"","Antwort bearbeiten",IF(G39&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G39,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E39&lt;&gt;"",IF(TODAY()&gt;=F39,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D39="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K39" s="2" t="n"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>13-Versandfertig-Mix</t>
+        </is>
+      </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Mix-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Akquise: 5 neue Leads Gewerbe & Büro (Schweißerei, Klavierstimmer, Vermessung, Versicherung, CPA)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2297,10 +2297,26 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>J.A.C. Welding &amp; Fabrication</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Schweißerei</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>jacwelding@sbcglobal.net</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3">
         <f>IF(OR(E40="",G40&lt;&gt;"",H40&lt;&gt;""),"",WORKDAY(E40,5))</f>
@@ -2314,13 +2330,33 @@
         <v/>
       </c>
       <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="n"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Accurate-Tune (Andy White)</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Klavierstimmer</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>andywhite@accurate-tune.com</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3">
         <f>IF(OR(E41="",G41&lt;&gt;"",H41&lt;&gt;""),"",WORKDAY(E41,5))</f>
@@ -2334,13 +2370,33 @@
         <v/>
       </c>
       <c r="K41" s="2" t="n"/>
-      <c r="L41" s="2" t="n"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>GSI Geomatic Solutions</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Landvermessung</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>shelby@gsisurvey.com</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3">
         <f>IF(OR(E42="",G42&lt;&gt;"",H42&lt;&gt;""),"",WORKDAY(E42,5))</f>
@@ -2354,13 +2410,33 @@
         <v/>
       </c>
       <c r="K42" s="2" t="n"/>
-      <c r="L42" s="2" t="n"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Armor Texas Insurance Agency</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Versicherung</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>hedy@armortexasins.com</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E43" s="3" t="n"/>
       <c r="F43" s="3">
         <f>IF(OR(E43="",G43&lt;&gt;"",H43&lt;&gt;""),"",WORKDAY(E43,5))</f>
@@ -2374,13 +2450,33 @@
         <v/>
       </c>
       <c r="K43" s="2" t="n"/>
-      <c r="L43" s="2" t="n"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Manjula P. Modi, CPA PLLC</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Steuerberater</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>info@fort-worth-cpa.com</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3">
         <f>IF(OR(E44="",G44&lt;&gt;"",H44&lt;&gt;""),"",WORKDAY(E44,5))</f>
@@ -2394,7 +2490,11 @@
         <v/>
       </c>
       <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>

</xml_diff>

<commit_message>
Gewerbe-Leads: Konzeptseiten fertig (Lead-Liste, Tracker)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2332,7 +2332,7 @@
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gewerbe-Leads: Projektnotizen, PDFs, Scroll-Videos und Ganzseiten-Bilder (J.A.C. Welding, Accurate-Tune, GSI, Armor Texas Insurance, Modi CPA)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2332,7 +2332,7 @@
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gewerbe-Leads: fünf Akquise-Mails vorbereitet (14-Versandfertig-Gewerbe), in den Projektnotizen, Tracker auf Versandbereit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2314,7 +2314,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E40" s="3" t="n"/>
@@ -2329,10 +2329,14 @@
         <f>IF(A40="","",IF(I40&lt;&gt;"","Antwort bearbeiten",IF(G40&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G40,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E40&lt;&gt;"",IF(TODAY()&gt;=F40,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D40="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K40" s="2" t="n"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>14-Versandfertig-Gewerbe</t>
+        </is>
+      </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2358,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E41" s="3" t="n"/>
@@ -2369,10 +2373,14 @@
         <f>IF(A41="","",IF(I41&lt;&gt;"","Antwort bearbeiten",IF(G41&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G41,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E41&lt;&gt;"",IF(TODAY()&gt;=F41,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D41="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K41" s="2" t="n"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>14-Versandfertig-Gewerbe</t>
+        </is>
+      </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2402,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E42" s="3" t="n"/>
@@ -2409,10 +2417,14 @@
         <f>IF(A42="","",IF(I42&lt;&gt;"","Antwort bearbeiten",IF(G42&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G42,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E42&lt;&gt;"",IF(TODAY()&gt;=F42,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D42="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K42" s="2" t="n"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>14-Versandfertig-Gewerbe</t>
+        </is>
+      </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2446,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E43" s="3" t="n"/>
@@ -2449,10 +2461,14 @@
         <f>IF(A43="","",IF(I43&lt;&gt;"","Antwort bearbeiten",IF(G43&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G43,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E43&lt;&gt;"",IF(TODAY()&gt;=F43,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D43="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K43" s="2" t="n"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>14-Versandfertig-Gewerbe</t>
+        </is>
+      </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2490,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E44" s="3" t="n"/>
@@ -2489,10 +2505,14 @@
         <f>IF(A44="","",IF(I44&lt;&gt;"","Antwort bearbeiten",IF(G44&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G44,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E44&lt;&gt;"",IF(TODAY()&gt;=F44,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D44="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K44" s="2" t="n"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>14-Versandfertig-Gewerbe</t>
+        </is>
+      </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Gewerbe-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: Mix-Mails und 5 Follow-ups verschickt (10.10.), Gewerbe-Mails und weitere Follow-ups im Zoho-Postausgang, KPS-Hinweis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -960,7 +960,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Abgeschickt</t>
+          <t>Follow-up gesendet</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -970,7 +970,9 @@
         <f>IF(OR(E9="",G9&lt;&gt;"",H9&lt;&gt;""),"",WORKDAY(E9,5))</f>
         <v/>
       </c>
-      <c r="G9" s="3" t="n"/>
+      <c r="G9" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="2">
@@ -982,7 +984,11 @@
           <t>07-Versandfertig-Structured-Foundation</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up 10.10. verschickt</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1002,7 +1008,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Abgeschickt</t>
+          <t>Follow-up gesendet</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -1012,7 +1018,9 @@
         <f>IF(OR(E10="",G10&lt;&gt;"",H10&lt;&gt;""),"",WORKDAY(E10,5))</f>
         <v/>
       </c>
-      <c r="G10" s="3" t="n"/>
+      <c r="G10" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="2">
@@ -1024,7 +1032,11 @@
           <t>08-Versandfertig-HVAC</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up 10.10. verschickt</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1044,7 +1056,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Abgeschickt</t>
+          <t>Follow-up gesendet</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -1054,7 +1066,9 @@
         <f>IF(OR(E11="",G11&lt;&gt;"",H11&lt;&gt;""),"",WORKDAY(E11,5))</f>
         <v/>
       </c>
-      <c r="G11" s="3" t="n"/>
+      <c r="G11" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n"/>
       <c r="J11" s="2">
@@ -1066,7 +1080,11 @@
           <t>08-Versandfertig-HVAC</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up 10.10. verschickt</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1086,7 +1104,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Abgeschickt</t>
+          <t>Follow-up gesendet</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -1096,7 +1114,9 @@
         <f>IF(OR(E12="",G12&lt;&gt;"",H12&lt;&gt;""),"",WORKDAY(E12,5))</f>
         <v/>
       </c>
-      <c r="G12" s="3" t="n"/>
+      <c r="G12" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n"/>
       <c r="J12" s="2">
@@ -1108,7 +1128,11 @@
           <t>08-Versandfertig-HVAC</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up 10.10. verschickt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1128,7 +1152,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Abgeschickt</t>
+          <t>Follow-up gesendet</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -1138,7 +1162,9 @@
         <f>IF(OR(E13="",G13&lt;&gt;"",H13&lt;&gt;""),"",WORKDAY(E13,5))</f>
         <v/>
       </c>
-      <c r="G13" s="3" t="n"/>
+      <c r="G13" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n"/>
       <c r="J13" s="2">
@@ -1150,7 +1176,11 @@
           <t>08-Versandfertig-HVAC</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up 10.10. verschickt</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1192,7 +1222,11 @@
           <t>09-Versandfertig-Architektur</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Follow-up liegt im Zoho-Postausgang (geplant)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1476,7 +1510,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1556,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>Erstmail am 10.10. erneut gesendet. Die alte Mail vom 09.10. liegt noch im Postausgang (Doppelversand vermeiden)</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1602,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1648,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1694,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1740,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1786,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1832,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1878,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>PDF angehängt; Scroll-Video erst nach einem Ja</t>
+          <t>PDF angehängt; Scroll-Video erst nach einem Ja; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1924,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Erstmail 09.10. mit PDF verschickt</t>
+          <t>Erstmail 09.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1970,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Erstmail 09.10. mit PDF verschickt</t>
+          <t>Erstmail 09.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -1982,7 +2016,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Erstmail 09.10. mit PDF verschickt</t>
+          <t>Erstmail 09.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2062,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Erstmail 09.10. mit PDF verschickt</t>
+          <t>Erstmail 09.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -2094,10 +2128,12 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F35" s="3">
         <f>IF(OR(E35="",G35&lt;&gt;"",H35&lt;&gt;""),"",WORKDAY(E35,5))</f>
         <v/>
@@ -2116,7 +2152,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail 10.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -2138,10 +2174,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F36" s="3">
         <f>IF(OR(E36="",G36&lt;&gt;"",H36&lt;&gt;""),"",WORKDAY(E36,5))</f>
         <v/>
@@ -2160,7 +2198,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail 10.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -2182,10 +2220,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F37" s="3">
         <f>IF(OR(E37="",G37&lt;&gt;"",H37&lt;&gt;""),"",WORKDAY(E37,5))</f>
         <v/>
@@ -2204,7 +2244,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail 10.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -2226,10 +2266,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F38" s="3">
         <f>IF(OR(E38="",G38&lt;&gt;"",H38&lt;&gt;""),"",WORKDAY(E38,5))</f>
         <v/>
@@ -2248,7 +2290,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail 10.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -2270,10 +2312,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F39" s="3">
         <f>IF(OR(E39="",G39&lt;&gt;"",H39&lt;&gt;""),"",WORKDAY(E39,5))</f>
         <v/>
@@ -2292,7 +2336,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail 10.10. mit PDF verschickt; Follow-up liegt im Zoho-Postausgang (geplant)</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2380,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2424,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2468,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2512,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2556,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
+          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Akquise: 5 neue Leads Läden & Dienste (Donuts, PC-Service, Schneiderei, Granit, Autopflege)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2561,10 +2561,26 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Funky Town Donuts</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Donut-Bäckerei</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>orders@funkytowndonuts.com</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3">
         <f>IF(OR(E45="",G45&lt;&gt;"",H45&lt;&gt;""),"",WORKDAY(E45,5))</f>
@@ -2578,13 +2594,33 @@
         <v/>
       </c>
       <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="n"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Michael's PC Sales &amp; Service</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Computer-Service</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>info@michaelspcsalesandservice.com</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E46" s="3" t="n"/>
       <c r="F46" s="3">
         <f>IF(OR(E46="",G46&lt;&gt;"",H46&lt;&gt;""),"",WORKDAY(E46,5))</f>
@@ -2598,13 +2634,33 @@
         <v/>
       </c>
       <c r="K46" s="2" t="n"/>
-      <c r="L46" s="2" t="n"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Helga's Custom Alterations</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Änderungsschneiderei</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>info@helgasalterations.com</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="3">
         <f>IF(OR(E47="",G47&lt;&gt;"",H47&lt;&gt;""),"",WORKDAY(E47,5))</f>
@@ -2618,13 +2674,33 @@
         <v/>
       </c>
       <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="n"/>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>DFW Granite</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Arbeitsplatten</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>dfwgranitetx@gmail.com</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E48" s="3" t="n"/>
       <c r="F48" s="3">
         <f>IF(OR(E48="",G48&lt;&gt;"",H48&lt;&gt;""),"",WORKDAY(E48,5))</f>
@@ -2638,13 +2714,33 @@
         <v/>
       </c>
       <c r="K48" s="2" t="n"/>
-      <c r="L48" s="2" t="n"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>DFW Auto Details</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Autopflege</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>dfwautodetails@gmail.com</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E49" s="3" t="n"/>
       <c r="F49" s="3">
         <f>IF(OR(E49="",G49&lt;&gt;"",H49&lt;&gt;""),"",WORKDAY(E49,5))</f>
@@ -2658,7 +2754,11 @@
         <v/>
       </c>
       <c r="K49" s="2" t="n"/>
-      <c r="L49" s="2" t="n"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>

</xml_diff>

<commit_message>
Läden-Leads: Konzeptseiten fertig (Lead-Liste, Tracker)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2596,7 +2596,7 @@
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2636,7 @@
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Läden-Leads: Projektnotizen, PDFs, Scroll-Videos und Ganzseiten-Bilder (Funky Town, Michael's PC, Helga's, DFW Granite, DFW Auto Details)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2596,7 +2596,7 @@
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2636,7 @@
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Läden-Leads: fünf Akquise-Mails vorbereitet (15-Versandfertig-Laden), in den Projektnotizen, Tracker auf Versandbereit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2578,7 +2578,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E45" s="3" t="n"/>
@@ -2593,10 +2593,14 @@
         <f>IF(A45="","",IF(I45&lt;&gt;"","Antwort bearbeiten",IF(G45&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G45,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E45&lt;&gt;"",IF(TODAY()&gt;=F45,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D45="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K45" s="2" t="n"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>15-Versandfertig-Laden</t>
+        </is>
+      </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2618,7 +2622,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E46" s="3" t="n"/>
@@ -2633,10 +2637,14 @@
         <f>IF(A46="","",IF(I46&lt;&gt;"","Antwort bearbeiten",IF(G46&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G46,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E46&lt;&gt;"",IF(TODAY()&gt;=F46,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D46="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K46" s="2" t="n"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>15-Versandfertig-Laden</t>
+        </is>
+      </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2666,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E47" s="3" t="n"/>
@@ -2673,10 +2681,14 @@
         <f>IF(A47="","",IF(I47&lt;&gt;"","Antwort bearbeiten",IF(G47&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G47,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E47&lt;&gt;"",IF(TODAY()&gt;=F47,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D47="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K47" s="2" t="n"/>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>15-Versandfertig-Laden</t>
+        </is>
+      </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2710,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E48" s="3" t="n"/>
@@ -2713,10 +2725,14 @@
         <f>IF(A48="","",IF(I48&lt;&gt;"","Antwort bearbeiten",IF(G48&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G48,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E48&lt;&gt;"",IF(TODAY()&gt;=F48,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D48="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K48" s="2" t="n"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>15-Versandfertig-Laden</t>
+        </is>
+      </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2754,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E49" s="3" t="n"/>
@@ -2753,10 +2769,14 @@
         <f>IF(A49="","",IF(I49&lt;&gt;"","Antwort bearbeiten",IF(G49&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G49,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E49&lt;&gt;"",IF(TODAY()&gt;=F49,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D49="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K49" s="2" t="n"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>15-Versandfertig-Laden</t>
+        </is>
+      </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF und Video fertig 10.10., Mail offen (Neue-Leads-Laden-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: Gewerbe-Mails und 6 Architektur-Mails am 10.10. verschickt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -1246,10 +1246,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F15" s="3">
         <f>IF(OR(E15="",G15&lt;&gt;"",H15&lt;&gt;""),"",WORKDAY(E15,5))</f>
         <v/>
@@ -1266,7 +1268,11 @@
           <t>09-Versandfertig-Architektur</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1286,10 +1292,12 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F16" s="3">
         <f>IF(OR(E16="",G16&lt;&gt;"",H16&lt;&gt;""),"",WORKDAY(E16,5))</f>
         <v/>
@@ -1306,7 +1314,11 @@
           <t>09-Versandfertig-Architektur</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1326,10 +1338,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F17" s="3">
         <f>IF(OR(E17="",G17&lt;&gt;"",H17&lt;&gt;""),"",WORKDAY(E17,5))</f>
         <v/>
@@ -1346,7 +1360,11 @@
           <t>09-Versandfertig-Architektur</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1366,10 +1384,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F18" s="3">
         <f>IF(OR(E18="",G18&lt;&gt;"",H18&lt;&gt;""),"",WORKDAY(E18,5))</f>
         <v/>
@@ -1386,7 +1406,11 @@
           <t>09-Versandfertig-Architektur</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1406,10 +1430,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F19" s="3">
         <f>IF(OR(E19="",G19&lt;&gt;"",H19&lt;&gt;""),"",WORKDAY(E19,5))</f>
         <v/>
@@ -1426,7 +1452,11 @@
           <t>09-Versandfertig-Architektur</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1446,10 +1476,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F20" s="3">
         <f>IF(OR(E20="",G20&lt;&gt;"",H20&lt;&gt;""),"",WORKDAY(E20,5))</f>
         <v/>
@@ -1466,7 +1498,11 @@
           <t>09-Versandfertig-Architektur</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2358,10 +2394,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F40" s="3">
         <f>IF(OR(E40="",G40&lt;&gt;"",H40&lt;&gt;""),"",WORKDAY(E40,5))</f>
         <v/>
@@ -2380,7 +2418,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
         </is>
       </c>
     </row>
@@ -2402,10 +2440,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F41" s="3">
         <f>IF(OR(E41="",G41&lt;&gt;"",H41&lt;&gt;""),"",WORKDAY(E41,5))</f>
         <v/>
@@ -2424,7 +2464,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
         </is>
       </c>
     </row>
@@ -2446,10 +2486,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F42" s="3">
         <f>IF(OR(E42="",G42&lt;&gt;"",H42&lt;&gt;""),"",WORKDAY(E42,5))</f>
         <v/>
@@ -2468,7 +2510,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
         </is>
       </c>
     </row>
@@ -2490,10 +2532,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F43" s="3">
         <f>IF(OR(E43="",G43&lt;&gt;"",H43&lt;&gt;""),"",WORKDAY(E43,5))</f>
         <v/>
@@ -2512,7 +2556,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
         </is>
       </c>
     </row>
@@ -2534,10 +2578,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Versandbereit</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="n"/>
+          <t>Abgeschickt</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="F44" s="3">
         <f>IF(OR(E44="",G44&lt;&gt;"",H44&lt;&gt;""),"",WORKDAY(E44,5))</f>
         <v/>
@@ -2556,7 +2602,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Erstmail mit PDF liegt im Zoho-Postausgang (geplant, Stand 10.10. noch nicht gesendet)</t>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Akquise: 5 neue Leads Umland & Freizeit (Hochzeitsort, Hundesalon, Plattenladen, Brauerei, Pest Weatherford)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2827,10 +2827,26 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>The Brooks at Weatherford</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Hochzeitsort</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>info@thebrooksatweatherford.com</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E50" s="3" t="n"/>
       <c r="F50" s="3">
         <f>IF(OR(E50="",G50&lt;&gt;"",H50&lt;&gt;""),"",WORKDAY(E50,5))</f>
@@ -2844,13 +2860,33 @@
         <v/>
       </c>
       <c r="K50" s="2" t="n"/>
-      <c r="L50" s="2" t="n"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Dog Grooming</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Mobiler Hundesalon</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>kdoby39@gmail.com</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E51" s="3" t="n"/>
       <c r="F51" s="3">
         <f>IF(OR(E51="",G51&lt;&gt;"",H51&lt;&gt;""),"",WORKDAY(E51,5))</f>
@@ -2864,13 +2900,33 @@
         <v/>
       </c>
       <c r="K51" s="2" t="n"/>
-      <c r="L51" s="2" t="n"/>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Doc's Records</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Plattenladen</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>daniel@docsrecords.com</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E52" s="3" t="n"/>
       <c r="F52" s="3">
         <f>IF(OR(E52="",G52&lt;&gt;"",H52&lt;&gt;""),"",WORKDAY(E52,5))</f>
@@ -2884,13 +2940,33 @@
         <v/>
       </c>
       <c r="K52" s="2" t="n"/>
-      <c r="L52" s="2" t="n"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>HopFusion Ale Works</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Brauerei</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>info@hopfusionaleworks.com</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E53" s="3" t="n"/>
       <c r="F53" s="3">
         <f>IF(OR(E53="",G53&lt;&gt;"",H53&lt;&gt;""),"",WORKDAY(E53,5))</f>
@@ -2904,13 +2980,33 @@
         <v/>
       </c>
       <c r="K53" s="2" t="n"/>
-      <c r="L53" s="2" t="n"/>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
-      <c r="D54" s="2" t="n"/>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Pitchford Pest Control</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Schädlingsbekämpfung</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>pitchfordpest@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E54" s="3" t="n"/>
       <c r="F54" s="3">
         <f>IF(OR(E54="",G54&lt;&gt;"",H54&lt;&gt;""),"",WORKDAY(E54,5))</f>
@@ -2924,7 +3020,11 @@
         <v/>
       </c>
       <c r="K54" s="2" t="n"/>
-      <c r="L54" s="2" t="n"/>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>

</xml_diff>

<commit_message>
Umland leads: concept pages built (Brooks, Mobile Dog Grooming, Doc's Records, HopFusion, Pitchford)
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2862,7 +2862,7 @@
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2902,7 @@
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Lead gefunden 10.10., Konzeptseite offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Umland leads: PDFs, scroll videos, project notes and prepared mails (16-Versandfertig-Umland)
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E50" s="3" t="n"/>
@@ -2859,10 +2859,14 @@
         <f>IF(A50="","",IF(I50&lt;&gt;"","Antwort bearbeiten",IF(G50&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G50,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E50&lt;&gt;"",IF(TODAY()&gt;=F50,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D50="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K50" s="2" t="n"/>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>16-Versandfertig-Umland</t>
+        </is>
+      </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2888,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E51" s="3" t="n"/>
@@ -2899,10 +2903,14 @@
         <f>IF(A51="","",IF(I51&lt;&gt;"","Antwort bearbeiten",IF(G51&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G51,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E51&lt;&gt;"",IF(TODAY()&gt;=F51,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D51="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K51" s="2" t="n"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>16-Versandfertig-Umland</t>
+        </is>
+      </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2932,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E52" s="3" t="n"/>
@@ -2939,10 +2947,14 @@
         <f>IF(A52="","",IF(I52&lt;&gt;"","Antwort bearbeiten",IF(G52&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G52,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E52&lt;&gt;"",IF(TODAY()&gt;=F52,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D52="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K52" s="2" t="n"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>16-Versandfertig-Umland</t>
+        </is>
+      </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2976,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E53" s="3" t="n"/>
@@ -2979,10 +2991,14 @@
         <f>IF(A53="","",IF(I53&lt;&gt;"","Antwort bearbeiten",IF(G53&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G53,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E53&lt;&gt;"",IF(TODAY()&gt;=F53,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D53="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K53" s="2" t="n"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>16-Versandfertig-Umland</t>
+        </is>
+      </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3020,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E54" s="3" t="n"/>
@@ -3019,10 +3035,14 @@
         <f>IF(A54="","",IF(I54&lt;&gt;"","Antwort bearbeiten",IF(G54&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G54,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E54&lt;&gt;"",IF(TODAY()&gt;=F54,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D54="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K54" s="2" t="n"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>16-Versandfertig-Umland</t>
+        </is>
+      </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 10.10., Mail/PDF/Video offen (Neue-Leads-Umland-2026-10-10)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 10.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Land & Handwerk leads (11.10.): Triple J Ranch Feed, RTM Ranch, Linda's Jewelry, Kar-Lynn Arts, Furniture & Upholstery Repair
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3047,10 +3047,26 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Triple J Ranch Feed Store</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Futtermittelladen</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>triplejranchfeeds@gmail.com</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E55" s="3" t="n"/>
       <c r="F55" s="3">
         <f>IF(OR(E55="",G55&lt;&gt;"",H55&lt;&gt;""),"",WORKDAY(E55,5))</f>
@@ -3064,13 +3080,33 @@
         <v/>
       </c>
       <c r="K55" s="2" t="n"/>
-      <c r="L55" s="2" t="n"/>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n"/>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>RTM Ranch Stables (Royal M Stables)</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Pferdestall &amp; Reitschule</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>rtmranch@ymail.com</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E56" s="3" t="n"/>
       <c r="F56" s="3">
         <f>IF(OR(E56="",G56&lt;&gt;"",H56&lt;&gt;""),"",WORKDAY(E56,5))</f>
@@ -3084,13 +3120,33 @@
         <v/>
       </c>
       <c r="K56" s="2" t="n"/>
-      <c r="L56" s="2" t="n"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n"/>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="n"/>
-      <c r="D57" s="2" t="n"/>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Linda's Jewelry</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Juwelier</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>lindasjewelrygold@gmail.com</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E57" s="3" t="n"/>
       <c r="F57" s="3">
         <f>IF(OR(E57="",G57&lt;&gt;"",H57&lt;&gt;""),"",WORKDAY(E57,5))</f>
@@ -3104,13 +3160,33 @@
         <v/>
       </c>
       <c r="K57" s="2" t="n"/>
-      <c r="L57" s="2" t="n"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="2" t="n"/>
-      <c r="D58" s="2" t="n"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Kar-Lynn Arts</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Bilderrahmen</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>karlynnarts@gmail.com</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E58" s="3" t="n"/>
       <c r="F58" s="3">
         <f>IF(OR(E58="",G58&lt;&gt;"",H58&lt;&gt;""),"",WORKDAY(E58,5))</f>
@@ -3124,13 +3200,33 @@
         <v/>
       </c>
       <c r="K58" s="2" t="n"/>
-      <c r="L58" s="2" t="n"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Furniture &amp; Upholstery Repair &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Möbelrestaurierung &amp; Polsterei</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>furniturerepair101@icloud.com</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E59" s="3" t="n"/>
       <c r="F59" s="3">
         <f>IF(OR(E59="",G59&lt;&gt;"",H59&lt;&gt;""),"",WORKDAY(E59,5))</f>
@@ -3144,7 +3240,11 @@
         <v/>
       </c>
       <c r="K59" s="2" t="n"/>
-      <c r="L59" s="2" t="n"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>

</xml_diff>

<commit_message>
vault backup: 2026-10-11 07:45:12
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3169,17 +3169,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Kar-Lynn Arts</t>
+          <t>Furniture &amp; Upholstery Repair &amp; Restoration</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Bilderrahmen</t>
+          <t>Möbelrestaurierung &amp; Polsterei</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>karlynnarts@gmail.com</t>
+          <t>furniturerepair101@icloud.com</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -3207,44 +3207,18 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Furniture &amp; Upholstery Repair &amp; Restoration</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Möbelrestaurierung &amp; Polsterei</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>furniturerepair101@icloud.com</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>In Bearbeitung</t>
-        </is>
-      </c>
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
       <c r="E59" s="3" t="n"/>
-      <c r="F59" s="3">
-        <f>IF(OR(E59="",G59&lt;&gt;"",H59&lt;&gt;""),"",WORKDAY(E59,5))</f>
-        <v/>
-      </c>
+      <c r="F59" s="3" t="n"/>
       <c r="G59" s="3" t="n"/>
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="2" t="n"/>
-      <c r="J59" s="2">
-        <f>IF(A59="","",IF(I59&lt;&gt;"","Antwort bearbeiten",IF(G59&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G59,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E59&lt;&gt;"",IF(TODAY()&gt;=F59,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D59="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
-        <v/>
-      </c>
+      <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
-        </is>
-      </c>
+      <c r="L59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>

</xml_diff>

<commit_message>
Land leads: Kar-Lynn Arts moved to reserve; concept pages built for Triple J, RTM Ranch, Linda's Jewelry, Furniture & Upholstery Repair
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3082,7 +3082,7 @@
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3122,7 @@
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       <c r="K57" s="2" t="n"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       <c r="K58" s="2" t="n"/>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Land-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Land leads: PDFs, scroll videos, project notes and prepared mails (17-Versandfertig-Land)
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E55" s="3" t="n"/>
@@ -3079,10 +3079,14 @@
         <f>IF(A55="","",IF(I55&lt;&gt;"","Antwort bearbeiten",IF(G55&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G55,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E55&lt;&gt;"",IF(TODAY()&gt;=F55,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D55="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K55" s="2" t="n"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>17-Versandfertig-Land</t>
+        </is>
+      </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3108,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E56" s="3" t="n"/>
@@ -3119,10 +3123,14 @@
         <f>IF(A56="","",IF(I56&lt;&gt;"","Antwort bearbeiten",IF(G56&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G56,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E56&lt;&gt;"",IF(TODAY()&gt;=F56,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D56="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K56" s="2" t="n"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>17-Versandfertig-Land</t>
+        </is>
+      </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3152,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E57" s="3" t="n"/>
@@ -3159,10 +3167,14 @@
         <f>IF(A57="","",IF(I57&lt;&gt;"","Antwort bearbeiten",IF(G57&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G57,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E57&lt;&gt;"",IF(TODAY()&gt;=F57,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D57="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K57" s="2" t="n"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>17-Versandfertig-Land</t>
+        </is>
+      </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3196,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E58" s="3" t="n"/>
@@ -3199,10 +3211,14 @@
         <f>IF(A58="","",IF(I58&lt;&gt;"","Antwort bearbeiten",IF(G58&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G58,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E58&lt;&gt;"",IF(TODAY()&gt;=F58,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D58="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K58" s="2" t="n"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>17-Versandfertig-Land</t>
+        </is>
+      </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite fertig 11.10., Mail/PDF/Video offen (Neue-Leads-Land-2026-10-11)</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Werkstatt leads (11.10.): Burleson Monuments, Fred Cheek Monuments, Malone Water Well, Mac's Marine, Harvest Moon Taxidermy
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3223,24 +3223,66 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Burleson Monuments</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Grabsteine &amp; Denkmäler</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>info@burlesonmonuments.com</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E59" s="3" t="n"/>
-      <c r="F59" s="3" t="n"/>
+      <c r="F59" s="3">
+        <f>IF(OR(E59="",G59&lt;&gt;"",H59&lt;&gt;""),"",WORKDAY(E59,5))</f>
+        <v/>
+      </c>
       <c r="G59" s="3" t="n"/>
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="2" t="n"/>
-      <c r="J59" s="2" t="n"/>
+      <c r="J59" s="2">
+        <f>IF(A59="","",IF(I59&lt;&gt;"","Antwort bearbeiten",IF(G59&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G59,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E59&lt;&gt;"",IF(TODAY()&gt;=F59,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D59="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
+        <v/>
+      </c>
       <c r="K59" s="2" t="n"/>
-      <c r="L59" s="2" t="n"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="n"/>
-      <c r="D60" s="2" t="n"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Fred Cheek Monuments</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Grabsteine &amp; Denkmäler</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>fcheek@fredcheekmonuments.com</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E60" s="3" t="n"/>
       <c r="F60" s="3">
         <f>IF(OR(E60="",G60&lt;&gt;"",H60&lt;&gt;""),"",WORKDAY(E60,5))</f>
@@ -3254,13 +3296,33 @@
         <v/>
       </c>
       <c r="K60" s="2" t="n"/>
-      <c r="L60" s="2" t="n"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
-      <c r="D61" s="2" t="n"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Malone Water Well Service &amp; Drilling</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Brunnenbohrer</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>malonewell@sbcglobal.net</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E61" s="3" t="n"/>
       <c r="F61" s="3">
         <f>IF(OR(E61="",G61&lt;&gt;"",H61&lt;&gt;""),"",WORKDAY(E61,5))</f>
@@ -3274,13 +3336,33 @@
         <v/>
       </c>
       <c r="K61" s="2" t="n"/>
-      <c r="L61" s="2" t="n"/>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Mac's Marine</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Bootsservice</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>macsmarinegranbury@gmail.com</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E62" s="3" t="n"/>
       <c r="F62" s="3">
         <f>IF(OR(E62="",G62&lt;&gt;"",H62&lt;&gt;""),"",WORKDAY(E62,5))</f>
@@ -3294,13 +3376,33 @@
         <v/>
       </c>
       <c r="K62" s="2" t="n"/>
-      <c r="L62" s="2" t="n"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
-      <c r="D63" s="2" t="n"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Harvest Moon Taxidermy</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Präparator</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>hmtaxidermy@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E63" s="3" t="n"/>
       <c r="F63" s="3">
         <f>IF(OR(E63="",G63&lt;&gt;"",H63&lt;&gt;""),"",WORKDAY(E63,5))</f>
@@ -3314,7 +3416,11 @@
         <v/>
       </c>
       <c r="K63" s="2" t="n"/>
-      <c r="L63" s="2" t="n"/>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>

</xml_diff>

<commit_message>
Werkstatt leads: concept pages, PDFs, scroll videos, project notes and prepared mails (18-Versandfertig-Werkstatt)
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3240,7 +3240,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E59" s="3" t="n"/>
@@ -3255,10 +3255,14 @@
         <f>IF(A59="","",IF(I59&lt;&gt;"","Antwort bearbeiten",IF(G59&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G59,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E59&lt;&gt;"",IF(TODAY()&gt;=F59,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D59="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K59" s="2" t="n"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>18-Versandfertig-Werkstatt</t>
+        </is>
+      </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3284,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E60" s="3" t="n"/>
@@ -3295,10 +3299,14 @@
         <f>IF(A60="","",IF(I60&lt;&gt;"","Antwort bearbeiten",IF(G60&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G60,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E60&lt;&gt;"",IF(TODAY()&gt;=F60,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D60="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K60" s="2" t="n"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>18-Versandfertig-Werkstatt</t>
+        </is>
+      </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3320,7 +3328,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E61" s="3" t="n"/>
@@ -3335,10 +3343,14 @@
         <f>IF(A61="","",IF(I61&lt;&gt;"","Antwort bearbeiten",IF(G61&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G61,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E61&lt;&gt;"",IF(TODAY()&gt;=F61,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D61="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K61" s="2" t="n"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>18-Versandfertig-Werkstatt</t>
+        </is>
+      </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3372,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E62" s="3" t="n"/>
@@ -3375,10 +3387,14 @@
         <f>IF(A62="","",IF(I62&lt;&gt;"","Antwort bearbeiten",IF(G62&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G62,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E62&lt;&gt;"",IF(TODAY()&gt;=F62,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D62="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K62" s="2" t="n"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>18-Versandfertig-Werkstatt</t>
+        </is>
+      </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3416,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E63" s="3" t="n"/>
@@ -3415,10 +3431,14 @@
         <f>IF(A63="","",IF(I63&lt;&gt;"","Antwort bearbeiten",IF(G63&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G63,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E63&lt;&gt;"",IF(TODAY()&gt;=F63,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D63="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K63" s="2" t="n"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>18-Versandfertig-Werkstatt</t>
+        </is>
+      </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Werkstatt-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Texas leads (11.10.): Kittner & Pate, Longview Body Shop, Pustka Family BBQ, RGF Insurance, Carmela Davis CPA
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3443,10 +3443,26 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
-      <c r="C64" s="2" t="n"/>
-      <c r="D64" s="2" t="n"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Kittner &amp; Pate Design Associates</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Architektur &amp; Innenarchitektur</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>jkittner@grandecom.net</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E64" s="3" t="n"/>
       <c r="F64" s="3">
         <f>IF(OR(E64="",G64&lt;&gt;"",H64&lt;&gt;""),"",WORKDAY(E64,5))</f>
@@ -3460,13 +3476,33 @@
         <v/>
       </c>
       <c r="K64" s="2" t="n"/>
-      <c r="L64" s="2" t="n"/>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n"/>
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="2" t="n"/>
-      <c r="D65" s="2" t="n"/>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Longview Body Shop (CPR)</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Unfall- &amp; Karosseriewerkstatt</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>kscoggins@longviewbodyshop.com</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E65" s="3" t="n"/>
       <c r="F65" s="3">
         <f>IF(OR(E65="",G65&lt;&gt;"",H65&lt;&gt;""),"",WORKDAY(E65,5))</f>
@@ -3480,13 +3516,33 @@
         <v/>
       </c>
       <c r="K65" s="2" t="n"/>
-      <c r="L65" s="2" t="n"/>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n"/>
-      <c r="B66" s="2" t="n"/>
-      <c r="C66" s="2" t="n"/>
-      <c r="D66" s="2" t="n"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Pustka Family Barbeque</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>BBQ-Restaurant</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>pustkafamilybbq@gmail.com</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E66" s="3" t="n"/>
       <c r="F66" s="3">
         <f>IF(OR(E66="",G66&lt;&gt;"",H66&lt;&gt;""),"",WORKDAY(E66,5))</f>
@@ -3500,13 +3556,33 @@
         <v/>
       </c>
       <c r="K66" s="2" t="n"/>
-      <c r="L66" s="2" t="n"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n"/>
-      <c r="B67" s="2" t="n"/>
-      <c r="C67" s="2" t="n"/>
-      <c r="D67" s="2" t="n"/>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>RGF Insurance Agency</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Versicherungsagentur</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>rgfinsag@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E67" s="3" t="n"/>
       <c r="F67" s="3">
         <f>IF(OR(E67="",G67&lt;&gt;"",H67&lt;&gt;""),"",WORKDAY(E67,5))</f>
@@ -3520,13 +3596,33 @@
         <v/>
       </c>
       <c r="K67" s="2" t="n"/>
-      <c r="L67" s="2" t="n"/>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n"/>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="2" t="n"/>
-      <c r="D68" s="2" t="n"/>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Carmela Davis, CPA, PLLC</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Steuerberatung (CPA)</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>cpa@cldcpa.com</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E68" s="3" t="n"/>
       <c r="F68" s="3">
         <f>IF(OR(E68="",G68&lt;&gt;"",H68&lt;&gt;""),"",WORKDAY(E68,5))</f>
@@ -3540,7 +3636,11 @@
         <v/>
       </c>
       <c r="K68" s="2" t="n"/>
-      <c r="L68" s="2" t="n"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>

</xml_diff>

<commit_message>
Texas leads: concept notes, PDFs, scroll videos and five prepared mails (19-Versandfertig-Texas); tracker rows 64-68 ready to send
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3460,7 +3460,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E64" s="3" t="n"/>
@@ -3475,10 +3475,14 @@
         <f>IF(A64="","",IF(I64&lt;&gt;"","Antwort bearbeiten",IF(G64&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G64,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E64&lt;&gt;"",IF(TODAY()&gt;=F64,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D64="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K64" s="2" t="n"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>19-Versandfertig-Texas</t>
+        </is>
+      </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3504,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E65" s="3" t="n"/>
@@ -3515,10 +3519,14 @@
         <f>IF(A65="","",IF(I65&lt;&gt;"","Antwort bearbeiten",IF(G65&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G65,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E65&lt;&gt;"",IF(TODAY()&gt;=F65,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D65="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K65" s="2" t="n"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>19-Versandfertig-Texas</t>
+        </is>
+      </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3548,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E66" s="3" t="n"/>
@@ -3555,10 +3563,14 @@
         <f>IF(A66="","",IF(I66&lt;&gt;"","Antwort bearbeiten",IF(G66&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G66,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E66&lt;&gt;"",IF(TODAY()&gt;=F66,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D66="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K66" s="2" t="n"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>19-Versandfertig-Texas</t>
+        </is>
+      </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3592,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E67" s="3" t="n"/>
@@ -3595,10 +3607,14 @@
         <f>IF(A67="","",IF(I67&lt;&gt;"","Antwort bearbeiten",IF(G67&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G67,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E67&lt;&gt;"",IF(TODAY()&gt;=F67,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D67="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K67" s="2" t="n"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>19-Versandfertig-Texas</t>
+        </is>
+      </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3636,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E68" s="3" t="n"/>
@@ -3635,10 +3651,14 @@
         <f>IF(A68="","",IF(I68&lt;&gt;"","Antwort bearbeiten",IF(G68&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G68,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E68&lt;&gt;"",IF(TODAY()&gt;=F68,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D68="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K68" s="2" t="n"/>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>19-Versandfertig-Texas</t>
+        </is>
+      </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2026-10-11), Konzeptseite offen</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Texas mails rewritten after the current rules in 01-Mailentwuerfe: one verified observation, 85-95 words, no attachment, offer a private preview link; delivery check first
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3482,7 +3482,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
+          <t>Mail neu nach Vorgaben in 01-Mailentwuerfe (11.10.): kein Anhang, Vorschau-Link anbieten. Erst Zustellung prüfen (SPF/DKIM/DMARC, Testmails), dann senden.</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
+          <t>Mail neu nach Vorgaben in 01-Mailentwuerfe (11.10.): kein Anhang, Vorschau-Link anbieten. Erst Zustellung prüfen (SPF/DKIM/DMARC, Testmails), dann senden.</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
+          <t>Mail neu nach Vorgaben in 01-Mailentwuerfe (11.10.): kein Anhang, Vorschau-Link anbieten. Erst Zustellung prüfen (SPF/DKIM/DMARC, Testmails), dann senden.</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
+          <t>Mail neu nach Vorgaben in 01-Mailentwuerfe (11.10.): kein Anhang, Vorschau-Link anbieten. Erst Zustellung prüfen (SPF/DKIM/DMARC, Testmails), dann senden.</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>Konzeptseite, PDF, Video und Mail fertig 11.10., versandbereit</t>
+          <t>Mail neu nach Vorgaben in 01-Mailentwuerfe (11.10.): kein Anhang, Vorschau-Link anbieten. Erst Zustellung prüfen (SPF/DKIM/DMARC, Testmails), dann senden.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
New leads Texas 2: five firms (Bannister Plumbing, The Flower Box, 4 Ever Green, Farmhouse 1905, Ted Coverage) plus reserve; tracker rows 69-73
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3663,10 +3663,26 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
-      <c r="D69" s="2" t="n"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Bannister Plumbing &amp; Air</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Klempner &amp; Klima</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>info@bannisterplumbing.com</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E69" s="3" t="n"/>
       <c r="F69" s="3">
         <f>IF(OR(E69="",G69&lt;&gt;"",H69&lt;&gt;""),"",WORKDAY(E69,5))</f>
@@ -3680,13 +3696,33 @@
         <v/>
       </c>
       <c r="K69" s="2" t="n"/>
-      <c r="L69" s="2" t="n"/>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n"/>
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="2" t="n"/>
-      <c r="D70" s="2" t="n"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>The Flower Box</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Blumenladen</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>tuitinc@sbcglobal.net</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E70" s="3" t="n"/>
       <c r="F70" s="3">
         <f>IF(OR(E70="",G70&lt;&gt;"",H70&lt;&gt;""),"",WORKDAY(E70,5))</f>
@@ -3700,13 +3736,33 @@
         <v/>
       </c>
       <c r="K70" s="2" t="n"/>
-      <c r="L70" s="2" t="n"/>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n"/>
-      <c r="B71" s="2" t="n"/>
-      <c r="C71" s="2" t="n"/>
-      <c r="D71" s="2" t="n"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>4 Ever Green Tree Care</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Baumpflege</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>4.evergreen.wftx@gmail.com</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E71" s="3" t="n"/>
       <c r="F71" s="3">
         <f>IF(OR(E71="",G71&lt;&gt;"",H71&lt;&gt;""),"",WORKDAY(E71,5))</f>
@@ -3720,13 +3776,33 @@
         <v/>
       </c>
       <c r="K71" s="2" t="n"/>
-      <c r="L71" s="2" t="n"/>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n"/>
-      <c r="B72" s="2" t="n"/>
-      <c r="C72" s="2" t="n"/>
-      <c r="D72" s="2" t="n"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Farmhouse 1905</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Hochzeitslocation</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>hello@farmhouse1905.com</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E72" s="3" t="n"/>
       <c r="F72" s="3">
         <f>IF(OR(E72="",G72&lt;&gt;"",H72&lt;&gt;""),"",WORKDAY(E72,5))</f>
@@ -3740,13 +3816,33 @@
         <v/>
       </c>
       <c r="K72" s="2" t="n"/>
-      <c r="L72" s="2" t="n"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n"/>
-      <c r="B73" s="2" t="n"/>
-      <c r="C73" s="2" t="n"/>
-      <c r="D73" s="2" t="n"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Ted Coverage</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Krankenversicherung (Agentur)</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>info@tedcoverage.com</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
       <c r="E73" s="3" t="n"/>
       <c r="F73" s="3">
         <f>IF(OR(E73="",G73&lt;&gt;"",H73&lt;&gt;""),"",WORKDAY(E73,5))</f>
@@ -3760,7 +3856,11 @@
         <v/>
       </c>
       <c r="K73" s="2" t="n"/>
-      <c r="L73" s="2" t="n"/>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>

</xml_diff>

<commit_message>
vault backup: 2026-10-11 13:59:41
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3705,17 +3705,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>The Flower Box</t>
+          <t>Weatherl &amp; Associates Architects</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Blumenladen</t>
+          <t>Architektur</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>tuitinc@sbcglobal.net</t>
+          <t>rickwaia@weatherl.net</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3738,7 +3738,7 @@
       <c r="K70" s="2" t="n"/>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+          <t>Ersatz für The Flower Box (Seite blockt Abrufe), Neue-Leads-Texas-2-2026-10-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Texas 2 leads: concept notes, PDFs, scroll videos and five mails after the current rules (20-Versandfertig-Texas-2); Weatherl replaces The Flower Box; tracker rows 69-73 ready to send after delivery check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -3680,7 +3680,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E69" s="3" t="n"/>
@@ -3695,10 +3695,14 @@
         <f>IF(A69="","",IF(I69&lt;&gt;"","Antwort bearbeiten",IF(G69&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G69,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E69&lt;&gt;"",IF(TODAY()&gt;=F69,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D69="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K69" s="2" t="n"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>20-Versandfertig-Texas-2</t>
+        </is>
+      </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10. (neue Vorgaben: kein Anhang, Vorschau-Link). Erst Zustellung prüfen, dann senden.</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3724,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E70" s="3" t="n"/>
@@ -3735,10 +3739,14 @@
         <f>IF(A70="","",IF(I70&lt;&gt;"","Antwort bearbeiten",IF(G70&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G70,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E70&lt;&gt;"",IF(TODAY()&gt;=F70,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D70="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K70" s="2" t="n"/>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>20-Versandfertig-Texas-2</t>
+        </is>
+      </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>Ersatz für The Flower Box (Seite blockt Abrufe), Neue-Leads-Texas-2-2026-10-11</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10. (neue Vorgaben: kein Anhang, Vorschau-Link). Erst Zustellung prüfen, dann senden.</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3768,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E71" s="3" t="n"/>
@@ -3775,10 +3783,14 @@
         <f>IF(A71="","",IF(I71&lt;&gt;"","Antwort bearbeiten",IF(G71&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G71,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E71&lt;&gt;"",IF(TODAY()&gt;=F71,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D71="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K71" s="2" t="n"/>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>20-Versandfertig-Texas-2</t>
+        </is>
+      </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10. (neue Vorgaben: kein Anhang, Vorschau-Link). Erst Zustellung prüfen, dann senden.</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3812,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E72" s="3" t="n"/>
@@ -3815,10 +3827,14 @@
         <f>IF(A72="","",IF(I72&lt;&gt;"","Antwort bearbeiten",IF(G72&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G72,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E72&lt;&gt;"",IF(TODAY()&gt;=F72,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D72="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K72" s="2" t="n"/>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>20-Versandfertig-Texas-2</t>
+        </is>
+      </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10. (neue Vorgaben: kein Anhang, Vorschau-Link). Erst Zustellung prüfen, dann senden.</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3856,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Versandbereit</t>
         </is>
       </c>
       <c r="E73" s="3" t="n"/>
@@ -3855,10 +3871,14 @@
         <f>IF(A73="","",IF(I73&lt;&gt;"","Antwort bearbeiten",IF(G73&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G73,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E73&lt;&gt;"",IF(TODAY()&gt;=F73,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D73="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K73" s="2" t="n"/>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>20-Versandfertig-Texas-2</t>
+        </is>
+      </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>Neuer Lead 11.10. (Neue-Leads-Texas-2-2026-10-11), wartet auf Freigabe</t>
+          <t>Konzeptseite, PDF, Video und Mail fertig 11.10. (neue Vorgaben: kein Anhang, Vorschau-Link). Erst Zustellung prüfen, dann senden.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Metallbau: Konzeptnotizen, Mails, Tracker; JAC Welding positive Antwort
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -2394,7 +2394,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Abgeschickt</t>
+          <t>Antwort erhalten</t>
         </is>
       </c>
       <c r="E40" s="3" t="n">
@@ -2405,8 +2405,14 @@
         <v/>
       </c>
       <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="2" t="n"/>
+      <c r="H40" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Positiv: möchte den Demo-Link</t>
+        </is>
+      </c>
       <c r="J40" s="2">
         <f>IF(A40="","",IF(I40&lt;&gt;"","Antwort bearbeiten",IF(G40&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G40,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E40&lt;&gt;"",IF(TODAY()&gt;=F40,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D40="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
@@ -2418,7 +2424,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet")</t>
+          <t>Erstmail 10.10. verschickt (laut Zoho "Gesendet") · 16.10.: positive Antwort, Demo-Link https://preview.northframesites.com/jac-welding-g3gcue/ (Antwort-Entwurf in northframe-outreach/messages.jsonl)</t>
         </is>
       </c>
     </row>
@@ -3883,10 +3889,26 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n"/>
-      <c r="B74" s="2" t="n"/>
-      <c r="C74" s="2" t="n"/>
-      <c r="D74" s="2" t="n"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Fabcon Industrial</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>sales@fabconindustrial.com</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E74" s="3" t="n"/>
       <c r="F74" s="3">
         <f>IF(OR(E74="",G74&lt;&gt;"",H74&lt;&gt;""),"",WORKDAY(E74,5))</f>
@@ -3899,14 +3921,38 @@
         <f>IF(A74="","",IF(I74&lt;&gt;"","Antwort bearbeiten",IF(G74&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G74,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E74&lt;&gt;"",IF(TODAY()&gt;=F74,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D74="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K74" s="2" t="n"/>
-      <c r="L74" s="2" t="n"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>21-Versandfertig-Metallbau</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Terminal Industries + Vorschau-Link fertig 16.10. (Neue-Leads-Metallbau-2026-10-16)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n"/>
-      <c r="B75" s="2" t="n"/>
-      <c r="C75" s="2" t="n"/>
-      <c r="D75" s="2" t="n"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Midwest Fab &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Metallbau &amp; Bau</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>sales@mwfcinc.com</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E75" s="3" t="n"/>
       <c r="F75" s="3">
         <f>IF(OR(E75="",G75&lt;&gt;"",H75&lt;&gt;""),"",WORKDAY(E75,5))</f>
@@ -3919,14 +3965,38 @@
         <f>IF(A75="","",IF(I75&lt;&gt;"","Antwort bearbeiten",IF(G75&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G75,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E75&lt;&gt;"",IF(TODAY()&gt;=F75,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D75="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K75" s="2" t="n"/>
-      <c r="L75" s="2" t="n"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>21-Versandfertig-Metallbau</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach The New Industrials + Vorschau-Link fertig 16.10. (Neue-Leads-Metallbau-2026-10-16)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n"/>
-      <c r="B76" s="2" t="n"/>
-      <c r="C76" s="2" t="n"/>
-      <c r="D76" s="2" t="n"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Amarillo Steel</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Schweißerei &amp; Maschinenbau</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>info@amarillosteel.com</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E76" s="3" t="n"/>
       <c r="F76" s="3">
         <f>IF(OR(E76="",G76&lt;&gt;"",H76&lt;&gt;""),"",WORKDAY(E76,5))</f>
@@ -3939,14 +4009,38 @@
         <f>IF(A76="","",IF(I76&lt;&gt;"","Antwort bearbeiten",IF(G76&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G76,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E76&lt;&gt;"",IF(TODAY()&gt;=F76,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D76="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K76" s="2" t="n"/>
-      <c r="L76" s="2" t="n"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>21-Versandfertig-Metallbau</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach "Craft, engineered." + Vorschau-Link fertig 16.10. (Neue-Leads-Metallbau-2026-10-16)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n"/>
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="2" t="n"/>
-      <c r="D77" s="2" t="n"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Brandon Welding &amp; Fabrication</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Schweißerei (Druckbehälter)</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>stewart@brandonwelding.com</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E77" s="3" t="n"/>
       <c r="F77" s="3">
         <f>IF(OR(E77="",G77&lt;&gt;"",H77&lt;&gt;""),"",WORKDAY(E77,5))</f>
@@ -3959,14 +4053,38 @@
         <f>IF(A77="","",IF(I77&lt;&gt;"","Antwort bearbeiten",IF(G77&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G77,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E77&lt;&gt;"",IF(TODAY()&gt;=F77,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D77="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K77" s="2" t="n"/>
-      <c r="L77" s="2" t="n"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>21-Versandfertig-Metallbau</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach AKT Oil Services + Vorschau-Link fertig 16.10. (Neue-Leads-Metallbau-2026-10-16)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n"/>
-      <c r="B78" s="2" t="n"/>
-      <c r="C78" s="2" t="n"/>
-      <c r="D78" s="2" t="n"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Vaquero Welding &amp; Fabrication</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Schweißerei &amp; Metallbau</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>robertd@vaquerowelding.com</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E78" s="3" t="n"/>
       <c r="F78" s="3">
         <f>IF(OR(E78="",G78&lt;&gt;"",H78&lt;&gt;""),"",WORKDAY(E78,5))</f>
@@ -3979,8 +4097,16 @@
         <f>IF(A78="","",IF(I78&lt;&gt;"","Antwort bearbeiten",IF(G78&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G78,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E78&lt;&gt;"",IF(TODAY()&gt;=F78,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D78="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K78" s="2" t="n"/>
-      <c r="L78" s="2" t="n"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>21-Versandfertig-Metallbau</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Bownds Ranches + Vorschau-Link fertig 16.10. (Neue-Leads-Metallbau-2026-10-16)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>

</xml_diff>

<commit_message>
Metallbau-2 leads: lead list, concept notes, PDFs, videos, mails, tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -4109,10 +4109,26 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n"/>
-      <c r="B79" s="2" t="n"/>
-      <c r="C79" s="2" t="n"/>
-      <c r="D79" s="2" t="n"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Texas Welding Company</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Stahlbau &amp; Schweißerei</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>sales@texasweldingcompany.com</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E79" s="3" t="n"/>
       <c r="F79" s="3">
         <f>IF(OR(E79="",G79&lt;&gt;"",H79&lt;&gt;""),"",WORKDAY(E79,5))</f>
@@ -4125,14 +4141,38 @@
         <f>IF(A79="","",IF(I79&lt;&gt;"","Antwort bearbeiten",IF(G79&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G79,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E79&lt;&gt;"",IF(TODAY()&gt;=F79,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D79="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K79" s="2" t="n"/>
-      <c r="L79" s="2" t="n"/>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>22-Versandfertig-Metallbau-2</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Summit Steel Works + Vorschau-Link, PDF, Video fertig 17.10. (Neue-Leads-Metallbau-2-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n"/>
-      <c r="B80" s="2" t="n"/>
-      <c r="C80" s="2" t="n"/>
-      <c r="D80" s="2" t="n"/>
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Ranchand Welding &amp; Fabrication</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Schweißerei (Pipeline, Öl &amp; Gas)</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>info@rhwfinc.com</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E80" s="3" t="n"/>
       <c r="F80" s="3">
         <f>IF(OR(E80="",G80&lt;&gt;"",H80&lt;&gt;""),"",WORKDAY(E80,5))</f>
@@ -4145,14 +4185,38 @@
         <f>IF(A80="","",IF(I80&lt;&gt;"","Antwort bearbeiten",IF(G80&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G80,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E80&lt;&gt;"",IF(TODAY()&gt;=F80,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D80="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K80" s="2" t="n"/>
-      <c r="L80" s="2" t="n"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>22-Versandfertig-Metallbau-2</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Kraken Industries + Vorschau-Link, PDF, Video fertig 17.10. (Neue-Leads-Metallbau-2-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n"/>
-      <c r="B81" s="2" t="n"/>
-      <c r="C81" s="2" t="n"/>
-      <c r="D81" s="2" t="n"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Texas Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Edelstahl-Metallbau (Großküchen)</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>nkey@texassheetmetal.com</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E81" s="3" t="n"/>
       <c r="F81" s="3">
         <f>IF(OR(E81="",G81&lt;&gt;"",H81&lt;&gt;""),"",WORKDAY(E81,5))</f>
@@ -4165,14 +4229,38 @@
         <f>IF(A81="","",IF(I81&lt;&gt;"","Antwort bearbeiten",IF(G81&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G81,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E81&lt;&gt;"",IF(TODAY()&gt;=F81,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D81="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K81" s="2" t="n"/>
-      <c r="L81" s="2" t="n"/>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>22-Versandfertig-Metallbau-2</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach MHB – Dutch Masters of Steel + Vorschau-Link, PDF, Video fertig 17.10. (Neue-Leads-Metallbau-2-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n"/>
-      <c r="B82" s="2" t="n"/>
-      <c r="C82" s="2" t="n"/>
-      <c r="D82" s="2" t="n"/>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>PFW Services</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Schweißerei &amp; Metallbau (Skids)</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Main@permianfabworks.com</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E82" s="3" t="n"/>
       <c r="F82" s="3">
         <f>IF(OR(E82="",G82&lt;&gt;"",H82&lt;&gt;""),"",WORKDAY(E82,5))</f>
@@ -4185,14 +4273,38 @@
         <f>IF(A82="","",IF(I82&lt;&gt;"","Antwort bearbeiten",IF(G82&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G82,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E82&lt;&gt;"",IF(TODAY()&gt;=F82,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D82="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K82" s="2" t="n"/>
-      <c r="L82" s="2" t="n"/>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>22-Versandfertig-Metallbau-2</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Structure Consulting Engineers + Vorschau-Link, PDF, Video fertig 17.10. (Neue-Leads-Metallbau-2-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n"/>
-      <c r="B83" s="2" t="n"/>
-      <c r="C83" s="2" t="n"/>
-      <c r="D83" s="2" t="n"/>
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Shadow Welding</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Schweißerei (Ölfeld)</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>info@shadowwelding.com</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E83" s="3" t="n"/>
       <c r="F83" s="3">
         <f>IF(OR(E83="",G83&lt;&gt;"",H83&lt;&gt;""),"",WORKDAY(E83,5))</f>
@@ -4205,8 +4317,16 @@
         <f>IF(A83="","",IF(I83&lt;&gt;"","Antwort bearbeiten",IF(G83&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G83,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E83&lt;&gt;"",IF(TODAY()&gt;=F83,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D83="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K83" s="2" t="n"/>
-      <c r="L83" s="2" t="n"/>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>22-Versandfertig-Metallbau-2</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Q Industrial + Vorschau-Link, PDF, Video fertig 17.10. (Neue-Leads-Metallbau-2-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>

</xml_diff>

<commit_message>
Pulverbeschichtung & CNC leads: lead list, concept notes, PDFs, videos, mail videos, mails with attachments, tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -4329,10 +4329,26 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n"/>
-      <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="n"/>
-      <c r="D84" s="2" t="n"/>
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Longhorn Powder Coating</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Pulverbeschichtung</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>longhornpowdercoat@sbcglobal.net</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E84" s="3" t="n"/>
       <c r="F84" s="3">
         <f>IF(OR(E84="",G84&lt;&gt;"",H84&lt;&gt;""),"",WORKDAY(E84,5))</f>
@@ -4345,14 +4361,38 @@
         <f>IF(A84="","",IF(I84&lt;&gt;"","Antwort bearbeiten",IF(G84&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G84,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E84&lt;&gt;"",IF(TODAY()&gt;=F84,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D84="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K84" s="2" t="n"/>
-      <c r="L84" s="2" t="n"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>23-Versandfertig-Pulverbeschichtung</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Paint It Easy, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Pulverbeschichtung-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n"/>
-      <c r="B85" s="2" t="n"/>
-      <c r="C85" s="2" t="n"/>
-      <c r="D85" s="2" t="n"/>
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>GTZ Powder Coating</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Pulverbeschichtung &amp; Auto-Styling</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>gtzpowdercoating@gmail.com</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E85" s="3" t="n"/>
       <c r="F85" s="3">
         <f>IF(OR(E85="",G85&lt;&gt;"",H85&lt;&gt;""),"",WORKDAY(E85,5))</f>
@@ -4365,14 +4405,38 @@
         <f>IF(A85="","",IF(I85&lt;&gt;"","Antwort bearbeiten",IF(G85&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G85,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E85&lt;&gt;"",IF(TODAY()&gt;=F85,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D85="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K85" s="2" t="n"/>
-      <c r="L85" s="2" t="n"/>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>23-Versandfertig-Pulverbeschichtung</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Zero Motorcycles, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Pulverbeschichtung-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n"/>
-      <c r="B86" s="2" t="n"/>
-      <c r="C86" s="2" t="n"/>
-      <c r="D86" s="2" t="n"/>
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Precision PowderCoat</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Pulverbeschichtung</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>info@ppcspring.com</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E86" s="3" t="n"/>
       <c r="F86" s="3">
         <f>IF(OR(E86="",G86&lt;&gt;"",H86&lt;&gt;""),"",WORKDAY(E86,5))</f>
@@ -4385,14 +4449,38 @@
         <f>IF(A86="","",IF(I86&lt;&gt;"","Antwort bearbeiten",IF(G86&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G86,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E86&lt;&gt;"",IF(TODAY()&gt;=F86,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D86="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K86" s="2" t="n"/>
-      <c r="L86" s="2" t="n"/>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>23-Versandfertig-Pulverbeschichtung</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Savic Motorcycles, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Pulverbeschichtung-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n"/>
-      <c r="B87" s="2" t="n"/>
-      <c r="C87" s="2" t="n"/>
-      <c r="D87" s="2" t="n"/>
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Fluid Industries</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Pulverbeschichtung, Cerakote, Hydro Dipping</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Wade@fluid-industries.com</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E87" s="3" t="n"/>
       <c r="F87" s="3">
         <f>IF(OR(E87="",G87&lt;&gt;"",H87&lt;&gt;""),"",WORKDAY(E87,5))</f>
@@ -4405,14 +4493,38 @@
         <f>IF(A87="","",IF(I87&lt;&gt;"","Antwort bearbeiten",IF(G87&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G87,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E87&lt;&gt;"",IF(TODAY()&gt;=F87,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D87="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K87" s="2" t="n"/>
-      <c r="L87" s="2" t="n"/>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>23-Versandfertig-Pulverbeschichtung</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Studio Ping Pong, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Pulverbeschichtung-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n"/>
-      <c r="B88" s="2" t="n"/>
-      <c r="C88" s="2" t="n"/>
-      <c r="D88" s="2" t="n"/>
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>CNC Mark</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>CNC-Werkstatt</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Mark@cnc-mark.com</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E88" s="3" t="n"/>
       <c r="F88" s="3">
         <f>IF(OR(E88="",G88&lt;&gt;"",H88&lt;&gt;""),"",WORKDAY(E88,5))</f>
@@ -4425,8 +4537,16 @@
         <f>IF(A88="","",IF(I88&lt;&gt;"","Antwort bearbeiten",IF(G88&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G88,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E88&lt;&gt;"",IF(TODAY()&gt;=F88,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D88="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K88" s="2" t="n"/>
-      <c r="L88" s="2" t="n"/>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>23-Versandfertig-Pulverbeschichtung</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Precision Calibration Systems, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Pulverbeschichtung-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>

</xml_diff>

<commit_message>
Kunstschmiede leads: lead list, concept notes, PDFs, videos, mail videos, mails with attachments, tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Vertrieb/Akquise-Tracker.xlsx
+++ b/03 Vertrieb/Akquise-Tracker.xlsx
@@ -4549,10 +4549,26 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n"/>
-      <c r="B89" s="2" t="n"/>
-      <c r="C89" s="2" t="n"/>
-      <c r="D89" s="2" t="n"/>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Oscar's Custom Iron Works</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>office@oscarsiron.com</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E89" s="3" t="n"/>
       <c r="F89" s="3">
         <f>IF(OR(E89="",G89&lt;&gt;"",H89&lt;&gt;""),"",WORKDAY(E89,5))</f>
@@ -4565,14 +4581,38 @@
         <f>IF(A89="","",IF(I89&lt;&gt;"","Antwort bearbeiten",IF(G89&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G89,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E89&lt;&gt;"",IF(TODAY()&gt;=F89,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D89="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K89" s="2" t="n"/>
-      <c r="L89" s="2" t="n"/>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>24-Versandfertig-Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Great Dane Furniture, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Kunstschmiede-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n"/>
-      <c r="B90" s="2" t="n"/>
-      <c r="C90" s="2" t="n"/>
-      <c r="D90" s="2" t="n"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>HCS MetalWorks / Ranchman Gates</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>hcstex@gmail.com</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E90" s="3" t="n"/>
       <c r="F90" s="3">
         <f>IF(OR(E90="",G90&lt;&gt;"",H90&lt;&gt;""),"",WORKDAY(E90,5))</f>
@@ -4585,14 +4625,38 @@
         <f>IF(A90="","",IF(I90&lt;&gt;"","Antwort bearbeiten",IF(G90&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G90,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E90&lt;&gt;"",IF(TODAY()&gt;=F90,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D90="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K90" s="2" t="n"/>
-      <c r="L90" s="2" t="n"/>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>24-Versandfertig-Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach James Bigley Ranches, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Kunstschmiede-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n"/>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
-      <c r="D91" s="2" t="n"/>
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>ATD Metalworks</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>atdmetalworks@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E91" s="3" t="n"/>
       <c r="F91" s="3">
         <f>IF(OR(E91="",G91&lt;&gt;"",H91&lt;&gt;""),"",WORKDAY(E91,5))</f>
@@ -4605,14 +4669,38 @@
         <f>IF(A91="","",IF(I91&lt;&gt;"","Antwort bearbeiten",IF(G91&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G91,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E91&lt;&gt;"",IF(TODAY()&gt;=F91,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D91="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K91" s="2" t="n"/>
-      <c r="L91" s="2" t="n"/>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>24-Versandfertig-Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Bownds Ranches, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Kunstschmiede-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n"/>
-      <c r="B92" s="2" t="n"/>
-      <c r="C92" s="2" t="n"/>
-      <c r="D92" s="2" t="n"/>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive Ironworks</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>rick@exclusiveironworks.com</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E92" s="3" t="n"/>
       <c r="F92" s="3">
         <f>IF(OR(E92="",G92&lt;&gt;"",H92&lt;&gt;""),"",WORKDAY(E92,5))</f>
@@ -4625,14 +4713,38 @@
         <f>IF(A92="","",IF(I92&lt;&gt;"","Antwort bearbeiten",IF(G92&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G92,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E92&lt;&gt;"",IF(TODAY()&gt;=F92,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D92="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K92" s="2" t="n"/>
-      <c r="L92" s="2" t="n"/>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>24-Versandfertig-Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach Gypsum Hills Ranch, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Kunstschmiede-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n"/>
-      <c r="B93" s="2" t="n"/>
-      <c r="C93" s="2" t="n"/>
-      <c r="D93" s="2" t="n"/>
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Smith Forge TX</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>eugenesmith2233@gmail.com</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Versandbereit</t>
+        </is>
+      </c>
       <c r="E93" s="3" t="n"/>
       <c r="F93" s="3">
         <f>IF(OR(E93="",G93&lt;&gt;"",H93&lt;&gt;""),"",WORKDAY(E93,5))</f>
@@ -4645,8 +4757,16 @@
         <f>IF(A93="","",IF(I93&lt;&gt;"","Antwort bearbeiten",IF(G93&lt;&gt;"",IF(TODAY()&gt;=WORKDAY(G93,7),"Als Keine Antwort abschließen","Warten auf Antwort"),IF(E93&lt;&gt;"",IF(TODAY()&gt;=F93,"Follow-up schreiben!","Warten bis Follow-up-Datum"),IF(D93="Versandbereit","Erstmail senden","Konzept fertigstellen")))))</f>
         <v/>
       </c>
-      <c r="K93" s="2" t="n"/>
-      <c r="L93" s="2" t="n"/>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>24-Versandfertig-Kunstschmiede</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>Konzeptseite nach La Forge du Malt, PDF + Mail-Video als Anhang, fertig 17.10. (Neue-Leads-Kunstschmiede-2026-10-17)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>

</xml_diff>